<commit_message>
Added a column for sample names
</commit_message>
<xml_diff>
--- a/sample_references.xlsx
+++ b/sample_references.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\CAS\Functional_Films\21_FF-EMEA\30-Technik_intern\01 Projekte Extrusion\2026\SIGMA-Project Dickenmessysteme\10 Project Basics\40 Produktportfolio u Ausfalldata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\costatf\Desktop\PolyGauge-NIR-Simulator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{64815218-F617-44A6-A36D-A0B6BD76296E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C81604F-53DF-49DC-9B32-4457461BE6D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E07CCF52-4D7A-450B-B28C-24700EBF0D94}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{E07CCF52-4D7A-450B-B28C-24700EBF0D94}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="49">
   <si>
     <t>SIGMA Project - Critical samples representative portfolio</t>
   </si>
@@ -160,6 +160,30 @@
   </si>
   <si>
     <t>layer composition, thickness, [µm] approx.</t>
+  </si>
+  <si>
+    <t>Sample Name</t>
+  </si>
+  <si>
+    <t>35 TPU/700 PET/65 TPU</t>
+  </si>
+  <si>
+    <t>PC (30)</t>
+  </si>
+  <si>
+    <t>PC (375)</t>
+  </si>
+  <si>
+    <t>PC (1000)</t>
+  </si>
+  <si>
+    <t>PC + TiO2 (620)</t>
+  </si>
+  <si>
+    <t>PC + Carbon (200)</t>
+  </si>
+  <si>
+    <t>PC + BaSO4 (400)</t>
   </si>
 </sst>
 </file>
@@ -276,7 +300,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -292,7 +316,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -608,19 +632,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8BE1A29-7AB6-4FAE-A35B-9FC0189ED5D9}">
-  <dimension ref="B2:G20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <dimension ref="B2:H20"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="6" max="6" width="18.42578125" customWidth="1"/>
-    <col min="7" max="7" width="25.140625" customWidth="1"/>
+    <col min="6" max="6" width="18.453125" customWidth="1"/>
+    <col min="7" max="7" width="25.1796875" customWidth="1"/>
+    <col min="8" max="8" width="23.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="23.25" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:8" ht="22.5" x14ac:dyDescent="0.45">
       <c r="B2" s="9" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:7" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:8" ht="39" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
@@ -639,16 +664,20 @@
       <c r="G3" s="1" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="H3" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B4" s="3"/>
       <c r="C4" s="4"/>
       <c r="D4" s="5"/>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
-    </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="H4" s="6"/>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="7" t="s">
         <v>6</v>
       </c>
@@ -667,8 +696,11 @@
       <c r="G5" s="7" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="H5" s="7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="7" t="s">
         <v>9</v>
       </c>
@@ -687,8 +719,11 @@
       <c r="G6" s="7" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="H6" s="7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="7" t="s">
         <v>12</v>
       </c>
@@ -707,8 +742,11 @@
       <c r="G7" s="7" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="H7" s="7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="7" t="s">
         <v>13</v>
       </c>
@@ -727,8 +765,11 @@
       <c r="G8" s="7" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="H8" s="7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" s="7" t="s">
         <v>14</v>
       </c>
@@ -747,8 +788,11 @@
       <c r="G9" s="7" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="H9" s="7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="7" t="s">
         <v>16</v>
       </c>
@@ -767,8 +811,11 @@
       <c r="G10" s="7" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="H10" s="7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" s="7" t="s">
         <v>18</v>
       </c>
@@ -787,8 +834,11 @@
       <c r="G11" s="7" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="H11" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" s="7" t="s">
         <v>20</v>
       </c>
@@ -807,8 +857,11 @@
       <c r="G12" s="7" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="H12" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" s="7" t="s">
         <v>22</v>
       </c>
@@ -827,8 +880,11 @@
       <c r="G13" s="7" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="H13" s="7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B14" s="7" t="s">
         <v>24</v>
       </c>
@@ -847,8 +903,11 @@
       <c r="G14" s="7" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="H14" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B15" s="7" t="s">
         <v>26</v>
       </c>
@@ -867,8 +926,11 @@
       <c r="G15" s="7" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="H15" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B16" s="7" t="s">
         <v>28</v>
       </c>
@@ -887,8 +949,11 @@
       <c r="G16" s="7" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="17" spans="2:7" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="H16" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" ht="25" x14ac:dyDescent="0.25">
       <c r="B17" s="7" t="s">
         <v>30</v>
       </c>
@@ -907,8 +972,11 @@
       <c r="G17" s="7" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="H17" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" s="7" t="s">
         <v>33</v>
       </c>
@@ -927,8 +995,11 @@
       <c r="G18" s="7" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="H18" s="7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B19" s="7" t="s">
         <v>36</v>
       </c>
@@ -947,8 +1018,11 @@
       <c r="G19" s="7" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="H19" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B20" s="7" t="s">
         <v>38</v>
       </c>
@@ -965,6 +1039,9 @@
         <v>7</v>
       </c>
       <c r="G20" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="H20" s="7" t="s">
         <v>39</v>
       </c>
     </row>

</xml_diff>